<commit_message>
Updated Dataset and Analytics
</commit_message>
<xml_diff>
--- a/outputs/evaluation_metrics.xlsx
+++ b/outputs/evaluation_metrics.xlsx
@@ -454,10 +454,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.775</v>
+        <v>0.813953488372093</v>
       </c>
       <c r="C2" t="n">
-        <v>77.5</v>
+        <v>81.3953488372093</v>
       </c>
     </row>
   </sheetData>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ36"/>
+  <dimension ref="A1:AM39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -627,25 +627,40 @@
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
+          <t>pred_person 40</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>pred_person 41</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>pred_person 42</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
           <t>pred_person 5</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>pred_person 6</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>pred_person 7</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>pred_person 8</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>pred_person 9</t>
         </is>
@@ -762,6 +777,15 @@
       <c r="AJ2" t="n">
         <v>0</v>
       </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -773,7 +797,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -830,7 +854,7 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
@@ -872,6 +896,15 @@
         <v>0</v>
       </c>
       <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -986,6 +1019,15 @@
       <c r="AJ4" t="n">
         <v>0</v>
       </c>
+      <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -1003,7 +1045,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1096,6 +1138,15 @@
         <v>0</v>
       </c>
       <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1210,6 +1261,15 @@
       <c r="AJ6" t="n">
         <v>0</v>
       </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1322,6 +1382,15 @@
       <c r="AJ7" t="n">
         <v>0</v>
       </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1434,6 +1503,15 @@
       <c r="AJ8" t="n">
         <v>0</v>
       </c>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1463,7 +1541,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -1544,6 +1622,15 @@
         <v>0</v>
       </c>
       <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1658,6 +1745,15 @@
       <c r="AJ10" t="n">
         <v>0</v>
       </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1770,6 +1866,15 @@
       <c r="AJ11" t="n">
         <v>0</v>
       </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1882,6 +1987,15 @@
       <c r="AJ12" t="n">
         <v>0</v>
       </c>
+      <c r="AK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1994,6 +2108,15 @@
       <c r="AJ13" t="n">
         <v>0</v>
       </c>
+      <c r="AK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -2008,7 +2131,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -2038,7 +2161,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -2104,6 +2227,15 @@
         <v>0</v>
       </c>
       <c r="AJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2156,7 +2288,7 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -2186,7 +2318,7 @@
         <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="n">
         <v>0</v>
@@ -2216,6 +2348,15 @@
         <v>0</v>
       </c>
       <c r="AJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2330,6 +2471,15 @@
       <c r="AJ16" t="n">
         <v>0</v>
       </c>
+      <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -2442,6 +2592,15 @@
       <c r="AJ17" t="n">
         <v>0</v>
       </c>
+      <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -2554,6 +2713,15 @@
       <c r="AJ18" t="n">
         <v>0</v>
       </c>
+      <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -2613,7 +2781,7 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -2664,6 +2832,15 @@
         <v>0</v>
       </c>
       <c r="AJ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2778,6 +2955,15 @@
       <c r="AJ20" t="n">
         <v>0</v>
       </c>
+      <c r="AK20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -2890,6 +3076,15 @@
       <c r="AJ21" t="n">
         <v>0</v>
       </c>
+      <c r="AK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -3002,6 +3197,15 @@
       <c r="AJ22" t="n">
         <v>0</v>
       </c>
+      <c r="AK22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -3114,6 +3318,15 @@
       <c r="AJ23" t="n">
         <v>0</v>
       </c>
+      <c r="AK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -3226,6 +3439,15 @@
       <c r="AJ24" t="n">
         <v>0</v>
       </c>
+      <c r="AK24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -3303,13 +3525,13 @@
         <v>0</v>
       </c>
       <c r="Y25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z25" t="n">
         <v>0</v>
       </c>
       <c r="AA25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB25" t="n">
         <v>0</v>
@@ -3336,6 +3558,15 @@
         <v>0</v>
       </c>
       <c r="AJ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3450,6 +3681,15 @@
       <c r="AJ26" t="n">
         <v>0</v>
       </c>
+      <c r="AK26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -3562,6 +3802,15 @@
       <c r="AJ27" t="n">
         <v>0</v>
       </c>
+      <c r="AK27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -3674,6 +3923,15 @@
       <c r="AJ28" t="n">
         <v>0</v>
       </c>
+      <c r="AK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -3712,7 +3970,7 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
         <v>0</v>
@@ -3736,7 +3994,7 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -3784,6 +4042,15 @@
         <v>0</v>
       </c>
       <c r="AJ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3898,6 +4165,15 @@
       <c r="AJ30" t="n">
         <v>0</v>
       </c>
+      <c r="AK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -4010,11 +4286,20 @@
       <c r="AJ31" t="n">
         <v>0</v>
       </c>
+      <c r="AK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>true_person 5</t>
+          <t>true_person 40</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -4120,13 +4405,22 @@
         <v>0</v>
       </c>
       <c r="AJ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>true_person 6</t>
+          <t>true_person 41</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -4232,13 +4526,22 @@
         <v>0</v>
       </c>
       <c r="AJ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>true_person 7</t>
+          <t>true_person 42</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -4338,19 +4641,28 @@
         <v>0</v>
       </c>
       <c r="AH34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI34" t="n">
         <v>0</v>
       </c>
       <c r="AJ34" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>true_person 8</t>
+          <t>true_person 5</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -4453,121 +4765,502 @@
         <v>0</v>
       </c>
       <c r="AI35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
+          <t>true_person 6</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>true_person 7</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>true_person 8</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" t="n">
+        <v>0</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
           <t>true_person 9</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>0</v>
-      </c>
-      <c r="R36" t="n">
-        <v>0</v>
-      </c>
-      <c r="S36" t="n">
-        <v>0</v>
-      </c>
-      <c r="T36" t="n">
-        <v>0</v>
-      </c>
-      <c r="U36" t="n">
-        <v>0</v>
-      </c>
-      <c r="V36" t="n">
-        <v>0</v>
-      </c>
-      <c r="W36" t="n">
-        <v>0</v>
-      </c>
-      <c r="X36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ36" t="n">
+      <c r="B39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM39" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4582,7 +5275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4638,13 +5331,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -4676,16 +5369,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -4761,7 +5454,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -4809,13 +5502,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -4847,13 +5540,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -4885,13 +5578,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C16" t="n">
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E16" t="n">
         <v>1</v>
@@ -4951,7 +5644,7 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -4961,13 +5654,13 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
         <v>0.5</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0.6666666666666666</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
@@ -5056,13 +5749,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
         <v>1</v>
@@ -5075,13 +5768,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
@@ -5094,13 +5787,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="C27" t="n">
         <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
@@ -5185,7 +5878,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>person 5</t>
+          <t>person 40</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -5204,7 +5897,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>person 6</t>
+          <t>person 41</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -5223,17 +5916,17 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>person 7</t>
+          <t>person 42</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
@@ -5242,7 +5935,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>person 8</t>
+          <t>person 5</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -5255,23 +5948,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>person 9</t>
+          <t>person 6</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
         <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="E36" t="n">
         <v>1</v>
@@ -5280,58 +5973,115 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>accuracy</t>
+          <t>person 7</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.775</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>0.775</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>0.775</v>
+        <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>0.775</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>macro avg</t>
+          <t>person 8</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>0.7571428571428571</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>0.7142857142857143</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
+          <t>person 9</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.813953488372093</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.813953488372093</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.813953488372093</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.813953488372093</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>macro avg</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.7368421052631579</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.7894736842105263</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.7535087719298247</v>
+      </c>
+      <c r="E41" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
           <t>weighted avg</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>0.725</v>
-      </c>
-      <c r="C39" t="n">
-        <v>0.775</v>
-      </c>
-      <c r="D39" t="n">
-        <v>0.7333333333333333</v>
-      </c>
-      <c r="E39" t="n">
-        <v>40</v>
+      <c r="B42" t="n">
+        <v>0.7596899224806201</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.813953488372093</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.7775193798449611</v>
+      </c>
+      <c r="E42" t="n">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>